<commit_message>
updated cleaning scripts to properly clean duckdb, added updated thesis.duckdb, updated weighting matrix code and ran code to generate cleaner weighting matrices
</commit_message>
<xml_diff>
--- a/2_SQL_database/Data_clean_updated/MCAS/Estados_US/Edos_USA_2010/ALABAMA_2010.xlsx
+++ b/2_SQL_database/Data_clean_updated/MCAS/Estados_US/Edos_USA_2010/ALABAMA_2010.xlsx
@@ -2760,7 +2760,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Gral. Simon Boivar</t>
+          <t>Gral. Simon Bolivar</t>
         </is>
       </c>
       <c r="C134">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Allende</t>
+          <t>San Miguel De Allende</t>
         </is>
       </c>
       <c r="C167">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>Dr. Arroyo</t>
+          <t>Doctor Arroyo</t>
         </is>
       </c>
       <c r="C522">
@@ -15342,7 +15342,7 @@
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>Yauhquemecan</t>
+          <t>Yauhquemehcan</t>
         </is>
       </c>
       <c r="C833">
@@ -16602,7 +16602,7 @@
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>Tuxpam</t>
+          <t>Tuxpan</t>
         </is>
       </c>
       <c r="C903">

</xml_diff>